<commit_message>
assign editors one update
</commit_message>
<xml_diff>
--- a/output/assigned_editors_one.xlsx
+++ b/output/assigned_editors_one.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H137"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1606,7 +1606,7 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Emily D’Arco</t>
+          <t>Vincient Arnold</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3051,28 +3051,28 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>India’s BRICS Moment: Power, Platforms, and Plural Order</t>
+          <t>Venezuela and U.S. Strategy</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>India’s BRICS Moment: Power, Platforms, and Plural Order.docx</t>
+          <t>Venezuela and U.S. Strategy.docx</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>geopolitics, international development</t>
+          <t>geopolitics, international security</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Vincient Arnold</t>
+          <t>Jonas Nepozitek</t>
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
@@ -3083,12 +3083,14 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Venezuela and U.S. Strategy</t>
+          <t xml:space="preserve">Losing the Narrative in Latin America:
+Disinformation, Great-Power Competition, and U.S. Strategy
+</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Venezuela and U.S. Strategy.docx</t>
+          <t>Losing the Narrative in Latin America: Disinformation, Great-Power Competition, and U.S. Strategy.docx</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3104,10 +3106,14 @@
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Jonas Nepozitek</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr"/>
+          <t>Alexandra Helfgott</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3115,37 +3121,35 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Losing the Narrative in Latin America:
-Disinformation, Great-Power Competition, and U.S. Strategy
-</t>
+          <t>Is Geopolitics ending IMF’s role as Lender of Last Resort?</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Losing the Narrative in Latin America: Disinformation, Great-Power Competition, and U.S. Strategy.docx</t>
+          <t>Is Geopolitics ending IMF’s role as Lender of Last Resort?.docx</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>geopolitics, international security</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr"/>
+          <t>geopolitics, united nations and multilateral institutions</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Alexandra Helfgott</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Jonas Nepozitek</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3153,32 +3157,28 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Is Geopolitics ending IMF’s role as Lender of Last Resort?</t>
+          <t>We Need Another Jonathan Larson. No Day, But Today</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Is Geopolitics ending IMF’s role as Lender of Last Resort?.docx</t>
+          <t>We Need Another Jonathan Larson. No Day, But Today..docx</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>geopolitics, united nations and multilateral institutions</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>cross-regional/global</t>
-        </is>
-      </c>
+          <t>global health</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Jonas Nepozitek</t>
+          <t>Rafael Gonzalez</t>
         </is>
       </c>
       <c r="H82" t="inlineStr"/>
@@ -3189,12 +3189,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>We Need Another Jonathan Larson. No Day, But Today</t>
+          <t xml:space="preserve">Men’s Silent Killer in the 21st Century: A Reflection on Men’s Mental Health Crisis </t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>We Need Another Jonathan Larson. No Day, But Today..docx</t>
+          <t>Men’s Silent Killer in the 21st Century: A Reflection on Men’s Mental Health Crisis .docx</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -3207,10 +3207,14 @@
           <t>global health</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Rafael Gonzalez</t>
+          <t>Rachel Lee</t>
         </is>
       </c>
       <c r="H83" t="inlineStr"/>
@@ -3221,32 +3225,28 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Men’s Silent Killer in the 21st Century: A Reflection on Men’s Mental Health Crisis </t>
+          <t>Potential of Tinospora cordifolia Stem Extract as a Natural Antimicrobial Agent Against Resistant Pathogens</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Men’s Silent Killer in the 21st Century: A Reflection on Men’s Mental Health Crisis .docx</t>
+          <t>Potential of Tinospora cordifolia Stem Extract as a Natural Antimicrobial Agent Against Resistant Pathogens.docx</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>global health</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>cross-regional/global</t>
-        </is>
-      </c>
+          <t>global health, other</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Rachel Lee</t>
+          <t>Michael Iwuoha</t>
         </is>
       </c>
       <c r="H84" t="inlineStr"/>
@@ -3257,28 +3257,28 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Potential of Tinospora cordifolia Stem Extract as a Natural Antimicrobial Agent Against Resistant Pathogens</t>
+          <t>Nation-Building in Bangladesh and the Global South: Why Internal Fractures, Not External Forces, Pose the Greatest Threat to Development</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Potential of Tinospora cordifolia Stem Extract as a Natural Antimicrobial Agent Against Resistant Pathogens.docx</t>
+          <t>Nation-Building in Bangladesh and the Global South.docx</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>global health, other</t>
+          <t>international development</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Michael Iwuoha</t>
+          <t>Gabriel Falk</t>
         </is>
       </c>
       <c r="H85" t="inlineStr"/>
@@ -3289,28 +3289,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Nation-Building in Bangladesh and the Global South: Why Internal Fractures, Not External Forces, Pose the Greatest Threat to Development</t>
+          <t xml:space="preserve">Revisiting M.V Xpress Pearl Accident
+</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Nation-Building in Bangladesh and the Global South.docx</t>
+          <t>Revisiting M.V Xpress Pearl Accident.docx</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>international development</t>
+          <t>international law</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Gabriel Falk</t>
+          <t>Lisa de Rafols</t>
         </is>
       </c>
       <c r="H86" t="inlineStr"/>
@@ -3321,29 +3322,32 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revisiting M.V Xpress Pearl Accident
-</t>
+          <t>The Quiet Threat to South Asia’s Most Important Treaty</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Revisiting M.V Xpress Pearl Accident.docx</t>
+          <t>The Quiet Threat to South Asia’s Most Important Treaty.docx</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>international law</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr"/>
+          <t>international law, united nations and multilateral institutions</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Lisa de Rafols</t>
+          <t>Kevin Chen</t>
         </is>
       </c>
       <c r="H87" t="inlineStr"/>
@@ -3354,32 +3358,28 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>The Quiet Threat to South Asia’s Most Important Treaty</t>
+          <t>The Paradox of Transparency: How Procedure Tames Personal Authority in the Epstein Files Fight</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>The Quiet Threat to South Asia’s Most Important Treaty.docx</t>
+          <t>The Paradox of Transparency: How Procedure Tames Personal Authority in the Epstein Files Fight.docx</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Op-ed</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>international law, united nations and multilateral institutions</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>south asia</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Kevin Chen</t>
+          <t>Alexandra Helfgott</t>
         </is>
       </c>
       <c r="H88" t="inlineStr"/>
@@ -3390,17 +3390,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>The Paradox of Transparency: How Procedure Tames Personal Authority in the Epstein Files Fight</t>
+          <t>When Sovereignty Fails: Foreign Intervention in Nigeria</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>The Paradox of Transparency: How Procedure Tames Personal Authority in the Epstein Files Fight.docx</t>
+          <t>When Sovereignty Fails: Foreign Intervention in Nigeria.docx</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Op-ed</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -3411,7 +3411,7 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Alexandra Helfgott</t>
+          <t>Sarah Cheung</t>
         </is>
       </c>
       <c r="H89" t="inlineStr"/>
@@ -3422,12 +3422,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>When Sovereignty Fails: Foreign Intervention in Nigeria</t>
+          <t>War, trauma and autobiography: An ecriture reading of Anne Frank’s Diary of a Young Girl</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>When Sovereignty Fails: Foreign Intervention in Nigeria.docx</t>
+          <t>War, trauma and autobiography: An ecriture reading of Anne Frank’s Diary of a Young Girl.docx</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -3454,12 +3454,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>War, trauma and autobiography: An ecriture reading of Anne Frank’s Diary of a Young Girl</t>
+          <t>Why Must We Be Commodified And Vulnerable? Unfolding Exploitation of the Female Body Under Capitalism Through Mieko Kawakwami's Breasts and Eggs</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>War, trauma and autobiography: An ecriture reading of Anne Frank’s Diary of a Young Girl.docx</t>
+          <t>Meiko_Kawakami_5_1.docx</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3475,7 +3475,7 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Sarah Cheung</t>
+          <t>Richard Ulbricht</t>
         </is>
       </c>
       <c r="H91" t="inlineStr"/>
@@ -3486,12 +3486,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Why Must We Be Commodified And Vulnerable? Unfolding Exploitation of the Female Body Under Capitalism Through Mieko Kawakwami's Breasts and Eggs</t>
+          <t>Psychopolitics of the “Good Indian Son”: Invisible Borders of Duty, Masculine Sacrifice, and the Hidden Cost to Families and Society</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Meiko_Kawakami_5_1.docx</t>
+          <t>Psychopolitics of the “Good Indian Son”: Invisible Borders of Duty, Masculine Sacrifice, and the Hidden Cost to Families and Society.docx</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -3507,7 +3507,7 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Richard Ulbricht</t>
+          <t>Mike Henry</t>
         </is>
       </c>
       <c r="H92" t="inlineStr"/>
@@ -3518,31 +3518,35 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Psychopolitics of the “Good Indian Son”: Invisible Borders of Duty, Masculine Sacrifice, and the Hidden Cost to Families and Society</t>
+          <t>Advancing Nigerian Women’s Digital and Entrepreneurial Skills: Prospects and Challenges</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Psychopolitics of the “Good Indian Son”: Invisible Borders of Duty, Masculine Sacrifice, and the Hidden Cost to Families and Society.docx</t>
+          <t>Advancing Nigerian Women’s Digital and Entrepreneurial Skills: Prospects and Challenges.docx</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>social innovation, other</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Mike Henry</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr"/>
+          <t>Alexandra Helfgott</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Other Category: Women and Skills</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3550,12 +3554,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Advancing Nigerian Women’s Digital and Entrepreneurial Skills: Prospects and Challenges</t>
+          <t>The End of State-Led Tech Governance</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Advancing Nigerian Women’s Digital and Entrepreneurial Skills: Prospects and Challenges.docx</t>
+          <t>The End of State-Led Tech Governance.docx</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3565,20 +3569,20 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>social innovation, other</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr"/>
+          <t>"technology, cybersecurity, and data governance", united nations and multilateral institutions</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Alexandra Helfgott</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>Other Category: Women and Skills</t>
-        </is>
-      </c>
+          <t>Emily D’Arco</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -3586,28 +3590,34 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>The End of State-Led Tech Governance</t>
+          <t xml:space="preserve">The Wages of Non-reciprocity:
+Evaluating India’s Neighbourhood First Policy
+</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>The End of State-Led Tech Governance.docx</t>
+          <t>The Wages of Non-reciprocity: Evaluating India’s Neighbourhood First Policy.docx</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>"technology, cybersecurity, and data governance", united nations and multilateral institutions</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr"/>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Rachel Lee</t>
+          <t>Lisa de Rafols</t>
         </is>
       </c>
       <c r="H95" t="inlineStr"/>
@@ -3618,30 +3628,32 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Wages of Non-reciprocity:
-Evaluating India’s Neighbourhood First Policy
-</t>
+          <t>Why Arctic Matters to India</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>The Wages of Non-reciprocity: Evaluating India’s Neighbourhood First Policy.docx</t>
+          <t>Why Arctic Matters to India.docx</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>"diplomacy, leadership, and foreign policy", geopolitics</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr"/>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics, international security</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Lisa de Rafols</t>
+          <t>Richard Ulbricht</t>
         </is>
       </c>
       <c r="H96" t="inlineStr"/>
@@ -3652,12 +3664,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Why Arctic Matters to India</t>
+          <t>When War Never Ends for Refugee Women</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Why Arctic Matters to India.docx</t>
+          <t>When War Never Ends for Refugee Women.docx</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3667,13 +3679,17 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>"diplomacy, leadership, and foreign policy", geopolitics, international security</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr"/>
+          <t>"human rights, humanitarian affairs, and global justice", "migration, refigees, and mobility"</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>central asia/eurasia</t>
+        </is>
+      </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Vincient Arnold</t>
+          <t>Rachel Lee</t>
         </is>
       </c>
       <c r="H97" t="inlineStr"/>
@@ -3684,28 +3700,32 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>When War Never Ends for Refugee Women</t>
+          <t>Breaking the Chains: Feminist Movements Against Patriarchy in Pakistan</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>When War Never Ends for Refugee Women.docx</t>
+          <t>Breaking the Chains: Feminist Movements Against Patriarchy in Pakistan.docx</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>"human rights, humanitarian affairs, and global justice", "migration, refigees, and mobility"</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr"/>
+          <t>"governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice", social innovation</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Emily D’Arco</t>
+          <t>Vincient Arnold</t>
         </is>
       </c>
       <c r="H98" t="inlineStr"/>
@@ -3716,12 +3736,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Breaking the Chains: Feminist Movements Against Patriarchy in Pakistan</t>
+          <t>Law as Strategy in Middle East Border Disputes</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Breaking the Chains: Feminist Movements Against Patriarchy in Pakistan.docx</t>
+          <t>Law as Strategy in Middle East Border Disputes.docx</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3731,10 +3751,14 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>"governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice", social innovation</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr"/>
+          <t>international law, "peace and conflict, peacebuilding"</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>middle east</t>
+        </is>
+      </c>
       <c r="G99" t="inlineStr">
         <is>
           <t>Catherine Dai</t>
@@ -3748,12 +3772,13 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Law as Strategy in Middle East Border Disputes</t>
+          <t xml:space="preserve">Cartographies of Exclusion on Unequal Terrain: Public Sector Data Regimes, Social Protection (or Lack Thereof), and Poor Governance in the Agrarian Regions of Northern Benin
+</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Law as Strategy in Middle East Border Disputes.docx</t>
+          <t>Cartographies of Exclusion on Unequal Terrain.docx</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3763,13 +3788,17 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>international law, "peace and conflict, peacebuilding"</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr"/>
+          <t>"governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice"</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>africa</t>
+        </is>
+      </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Rachel Lee</t>
+          <t>Sarah Cheung</t>
         </is>
       </c>
       <c r="H100" t="inlineStr"/>
@@ -3780,13 +3809,13 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cartographies of Exclusion on Unequal Terrain: Public Sector Data Regimes, Social Protection (or Lack Thereof), and Poor Governance in the Agrarian Regions of Northern Benin
-</t>
+          <t>How WHO Can Improve Its 2025 Amendment:
+The Global Pandemic Patent Fund</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Cartographies of Exclusion on Unequal Terrain.docx</t>
+          <t>How WHO Can Improve Its 2025 Amendment: The Global Pandemic Patent Fund.docx</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -3796,13 +3825,17 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>"governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice"</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr"/>
+          <t>global health, united nations and multilateral institutions</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Gabriel Falk</t>
+          <t>Emily D’Arco</t>
         </is>
       </c>
       <c r="H101" t="inlineStr"/>
@@ -3813,13 +3846,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>How WHO Can Improve Its 2025 Amendment:
-The Global Pandemic Patent Fund</t>
+          <t>Selective Multilateralism in Outer Space: Daisy-Chain Diplomacy and the Crisis of Peaceful Purposes</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>How WHO Can Improve Its 2025 Amendment: The Global Pandemic Patent Fund.docx</t>
+          <t>Selective Multilateralism in Outer Space: Daisy-Chain Diplomacy and the Crisis of Peaceful Purposes.docx</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -3829,13 +3861,17 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>global health, united nations and multilateral institutions</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr"/>
+          <t>"diplomacy, leadership, and foreign policy", international law, international security, "peace and conflict, peacebuilding"</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Jacob Coughlin</t>
+          <t>Lisa de Rafols</t>
         </is>
       </c>
       <c r="H102" t="inlineStr"/>
@@ -3846,12 +3882,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Selective Multilateralism in Outer Space: Daisy-Chain Diplomacy and the Crisis of Peaceful Purposes</t>
+          <t>Hares &amp; Hounds: How Do the EMDEs Utilize the WTO Paralysis?</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Selective Multilateralism in Outer Space: Daisy-Chain Diplomacy and the Crisis of Peaceful Purposes.docx</t>
+          <t>Hares &amp; Hounds: How Do the EMDEs Utilize the WTO Paralysis?.docx</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3861,13 +3897,17 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>"diplomacy, leadership, and foreign policy", international law, international security, "peace and conflict, peacebuilding"</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr"/>
+          <t>"global economy, finance, and trade", international development, united nations and multilateral institutions</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Sarah Cheung</t>
+          <t>Gabriel Falk</t>
         </is>
       </c>
       <c r="H103" t="inlineStr"/>
@@ -3878,12 +3918,13 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Hares &amp; Hounds: How Do the EMDEs Utilize the WTO Paralysis?</t>
+          <t xml:space="preserve">Darija: The Missing Piece in Morocco’s Education Reform
+</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Hares &amp; Hounds: How Do the EMDEs Utilize the WTO Paralysis?.docx</t>
+          <t>Darija: The Missing Piece in Morocco’s Education Reform.docx</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3893,13 +3934,17 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>"global economy, finance, and trade", international development, united nations and multilateral institutions</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr"/>
+          <t>international development, other</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>africa</t>
+        </is>
+      </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Lisa de Rafols</t>
+          <t>Michael Iwuoha</t>
         </is>
       </c>
       <c r="H104" t="inlineStr"/>
@@ -3910,13 +3955,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Darija: The Missing Piece in Morocco’s Education Reform
-</t>
+          <t>A World Up for Grabs: How MSC 2025 Reveals the Erosion of U.S. Dominance</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Darija: The Missing Piece in Morocco’s Education Reform.docx</t>
+          <t>A World Up for Grabs: How MSC 2025 Reveals the Erosion of U.S. Dominance.docx</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -3926,13 +3970,17 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>international development, other</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr"/>
+          <t>international security, united nations and multilateral institutions</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Richard Ulbricht</t>
+          <t>Jacob Coughlin</t>
         </is>
       </c>
       <c r="H105" t="inlineStr"/>
@@ -3943,25 +3991,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>A World Up for Grabs: How MSC 2025 Reveals the Erosion of U.S. Dominance</t>
+          <t>Bangladesh’s Delta Plan 2100 as Climate Diplomacy</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>A World Up for Grabs: How MSC 2025 Reveals the Erosion of U.S. Dominance.docx</t>
+          <t>Bangladesh’s Delta Plan 2100 as Climate Diplomacy.docx</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>international security, united nations and multilateral institutions</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr"/>
+          <t>"climate, energy, and sustainability", international development</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
       <c r="G106" t="inlineStr">
         <is>
           <t>Rafael Gonzalez</t>
@@ -3975,28 +4027,32 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Bangladesh’s Delta Plan 2100 as Climate Diplomacy</t>
+          <t>From Delhi to London, Brussels and Sydney: The Worldwide Shift From Violent Extremists to White-Collar Terror Facilitators</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Bangladesh’s Delta Plan 2100 as Climate Diplomacy.docx</t>
+          <t>From Delhi to London, Brussels and Sydney: The Worldwide Shift From Violent Extremists to White-Collar Terror Facilitators.docx</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>"climate, energy, and sustainability", international development</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr"/>
+          <t>geopolitics, international security, "peace and conflict, peacebuilding"</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Vincient Arnold</t>
+          <t>Rachel Lee</t>
         </is>
       </c>
       <c r="H107" t="inlineStr"/>
@@ -4007,12 +4063,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>From Delhi to London, Brussels and Sydney: The Worldwide Shift From Violent Extremists to White-Collar Terror Facilitators</t>
+          <t>AI and Climate Resilience in Pakistan - Harnessing technology for sustainable policy solutions</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>From Delhi to London, Brussels and Sydney: The Worldwide Shift From Violent Extremists to White-Collar Terror Facilitators.docx</t>
+          <t>AI and Climate Resilience in Pakistan - Harnessing technology for sustainable policy solutions.doc</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -4022,13 +4078,17 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>geopolitics, international security, "peace and conflict, peacebuilding"</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr"/>
+          <t>"climate, energy, and sustainability"</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Emily D’Arco</t>
+          <t>Richard Ulbricht</t>
         </is>
       </c>
       <c r="H108" t="inlineStr"/>
@@ -4039,12 +4099,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>AI and Climate Resilience in Pakistan - Harnessing technology for sustainable policy solutions</t>
+          <t>Binding Force of Inter-American Court Judgements, Conventionality Control and Constitutional Adjudication: Reflection Prompted by President Pacheco’s Remarks</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>AI and Climate Resilience in Pakistan - Harnessing technology for sustainable policy solutions.doc</t>
+          <t>Binding Force of Inter-American Court Judgements, Conventionality Control and Constitutional Adjudication: Reflection Prompted by President Pacheco’s Remarks.docx</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -4054,13 +4114,17 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>"climate, energy, and sustainability"</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr"/>
+          <t>"human rights, humanitarian affairs, and global justice", international law</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>latin america</t>
+        </is>
+      </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Jonas Nepozitek</t>
+          <t>Sarah Cheung</t>
         </is>
       </c>
       <c r="H109" t="inlineStr"/>
@@ -4071,12 +4135,13 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Binding Force of Inter-American Court Judgements, Conventionality Control and Constitutional Adjudication: Reflection Prompted by President Pacheco’s Remarks</t>
+          <t xml:space="preserve">Does U.S. foreign policy become more performative?
+</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Binding Force of Inter-American Court Judgements, Conventionality Control and Constitutional Adjudication: Reflection Prompted by President Pacheco’s Remarks.docx</t>
+          <t>Does U.S. foreign policy become more performative?.docx</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -4086,10 +4151,14 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>"human rights, humanitarian affairs, and global justice", international law</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr"/>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>north america</t>
+        </is>
+      </c>
       <c r="G110" t="inlineStr">
         <is>
           <t>Kevin Chen</t>
@@ -4103,13 +4172,13 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Does U.S. foreign policy become more performative?
+          <t xml:space="preserve">America’s AI Debate Is Blinding Us to China’s Actual Approach to AI 
 </t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Does U.S. foreign policy become more performative?.docx</t>
+          <t>America’s AI Debate Is Blinding Us to China’s Actual Approach to AI .docx</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -4119,13 +4188,18 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>"diplomacy, leadership, and foreign policy", geopolitics</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr"/>
+          <t>geopolitics, "technology, cybersecurity, and data governance"</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>east asia
+north america</t>
+        </is>
+      </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Mike Henry</t>
+          <t>Vincient Arnold</t>
         </is>
       </c>
       <c r="H111" t="inlineStr"/>
@@ -4136,13 +4210,14 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">America’s AI Debate Is Blinding Us to China’s Actual Approach to AI 
+          <t xml:space="preserve">Lone Star Statecraft:
+Sub-national Diplomacy in Texas-Israel Relations
 </t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>America’s AI Debate Is Blinding Us to China’s Actual Approach to AI .docx</t>
+          <t>Lone Star Statecraft: Sub-national Diplomacy in Texas-Israel Relations.docx</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -4152,13 +4227,17 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>geopolitics, "technology, cybersecurity, and data governance"</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr"/>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Catherine Dai</t>
+          <t>Emily D’Arco</t>
         </is>
       </c>
       <c r="H112" t="inlineStr"/>
@@ -4169,14 +4248,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lone Star Statecraft:
-Sub-national Diplomacy in Texas-Israel Relations
-</t>
+          <t xml:space="preserve">From Cotton to Chips: Taiwan’s Silicon Shield and the Perils of Economic Deterrence </t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Lone Star Statecraft: Sub-national Diplomacy in Texas-Israel Relations.docx</t>
+          <t>From Cotton to Chips: Taiwan’s Silicon Shield and the Perils of Economic Deterrence (2300 words).docx</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -4186,13 +4263,17 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>"diplomacy, leadership, and foreign policy", geopolitics</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr"/>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics, international security</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>east asia</t>
+        </is>
+      </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Michael Iwuoha</t>
+          <t>Catherine Dai</t>
         </is>
       </c>
       <c r="H113" t="inlineStr"/>
@@ -4203,12 +4284,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">From Cotton to Chips: Taiwan’s Silicon Shield and the Perils of Economic Deterrence </t>
+          <t>Stealth Sovereignty: The Strategic Imperative of the Indo-Russian Su-57 Ecosystem</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>From Cotton to Chips: Taiwan’s Silicon Shield and the Perils of Economic Deterrence (2300 words).docx</t>
+          <t>Stealth Sovereignty: The Strategic Imperative of the Indo-Russian Su-57 Ecosystem.docx</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -4218,13 +4299,17 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>"diplomacy, leadership, and foreign policy", geopolitics, international security</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr"/>
+          <t>geopolitics</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Rachel Lee</t>
+          <t>Jonas Nepozitek</t>
         </is>
       </c>
       <c r="H114" t="inlineStr"/>
@@ -4235,28 +4320,32 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Stealth Sovereignty: The Strategic Imperative of the Indo-Russian Su-57 Ecosystem</t>
+          <t>When Sanctions Hit the Wrong Target: Why International Economic Pressure on Iran Demands Distributional Impact Assessment</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Stealth Sovereignty: The Strategic Imperative of the Indo-Russian Su-57 Ecosystem.docx</t>
+          <t>When Sanctions Hit the Wrong Target: Why International Economic Pressure on Iran Demands Distributional Impact Assessment.docx</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>geopolitics</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr"/>
+          <t>geopolitics, "global economy, finance, and trade", "governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice"</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>middle east</t>
+        </is>
+      </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Jacob Coughlin</t>
+          <t>Catherine Dai</t>
         </is>
       </c>
       <c r="H115" t="inlineStr"/>
@@ -4267,28 +4356,32 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>When Sanctions Hit the Wrong Target: Why International Economic Pressure on Iran Demands Distributional Impact Assessment</t>
+          <t xml:space="preserve">Environmental Justice Struggles and Neoliberal Intervention in Access to Sustainable Housing of Marginalised Communities </t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>When Sanctions Hit the Wrong Target: Why International Economic Pressure on Iran Demands Distributional Impact Assessment.docx</t>
+          <t>Environmental Justice Struggles and Neoliberal Intervention in Access to Sustainable Housing of Marginalised Communities .docx</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>geopolitics, "global economy, finance, and trade", "governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice"</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Gabriel Falk</t>
+          <t>Mike Henry</t>
         </is>
       </c>
       <c r="H116" t="inlineStr"/>
@@ -4299,28 +4392,32 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Environmental Justice Struggles and Neoliberal Intervention in Access to Sustainable Housing of Marginalised Communities </t>
+          <t>Digitally Empowered India: What Lessons Can Be Learned from India’s Tech Boom?</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Environmental Justice Struggles and Neoliberal Intervention in Access to Sustainable Housing of Marginalised Communities .docx</t>
+          <t>Digitally Empowered India: What Lessons Can Be Learned from India’s Tech Boom?.docx</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr"/>
+          <t>"technology, cybersecurity, and data governance"</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Sarah Cheung</t>
+          <t>Lisa de Rafols</t>
         </is>
       </c>
       <c r="H117" t="inlineStr"/>
@@ -4331,28 +4428,32 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Digitally Empowered India: What Lessons Can Be Learned from India’s Tech Boom?</t>
+          <t>The Role of the International Organization for Migration in Supporting Indonesia's Refugee Governance 2020-2024</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Digitally Empowered India: What Lessons Can Be Learned from India’s Tech Boom?.docx</t>
+          <t>The Role of the International Organization for Migration in Supporting Indonesia's Refugee Governance 2020-2024.docx</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>"technology, cybersecurity, and data governance"</t>
-        </is>
-      </c>
-      <c r="F118" t="inlineStr"/>
+          <t>"diplomacy, leadership, and foreign policy", "governance, democracy, and institutions", "migration, refigees, and mobility"</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>southeast asia</t>
+        </is>
+      </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Lisa de Rafols</t>
+          <t>Gabriel Falk</t>
         </is>
       </c>
       <c r="H118" t="inlineStr"/>
@@ -4363,28 +4464,32 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>The Role of the International Organization for Migration in Supporting Indonesia's Refugee Governance 2020-2024</t>
+          <t>Book Reviews - "As Long as the Lemon Trees Grow" &amp; "The Terror"</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>The Role of the International Organization for Migration in Supporting Indonesia's Refugee Governance 2020-2024.docx</t>
+          <t>Book Reviews - "As Long as the Lemon Trees Grow" &amp; "The Terror".docx</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Book Review</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>"diplomacy, leadership, and foreign policy", "governance, democracy, and institutions", "migration, refigees, and mobility"</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>middle east</t>
+        </is>
+      </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Richard Ulbricht</t>
+          <t>Michael Iwuoha</t>
         </is>
       </c>
       <c r="H119" t="inlineStr"/>
@@ -4395,28 +4500,32 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Book Reviews - "As Long as the Lemon Trees Grow" &amp; "The Terror"</t>
+          <t>Within the Empire of Code: Poetry and the Borderless Ascendancy of Artificial Intelligence</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Book Reviews - "As Long as the Lemon Trees Grow" &amp; "The Terror".docx</t>
+          <t>Within the Empire of Code: Poetry and the Borderless Ascendancy of Artificial Intelligence.doc</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Book Review</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr"/>
+          <t>geopolitics, "peace and conflict, peacebuilding", "technology, cybersecurity, and data governance", other</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Rafael Gonzalez</t>
+          <t>Jacob Coughlin</t>
         </is>
       </c>
       <c r="H120" t="inlineStr"/>
@@ -4427,28 +4536,32 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Within the Empire of Code: Poetry and the Borderless Ascendancy of Artificial Intelligence</t>
+          <t>At the Edge of Three Borders</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Within the Empire of Code: Poetry and the Borderless Ascendancy of Artificial Intelligence.doc</t>
+          <t>At the Edge of Three Borders.docx</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Photo Essay</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>geopolitics, "peace and conflict, peacebuilding", "technology, cybersecurity, and data governance", other</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr"/>
+          <t>geopolitics, international security</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>middle east</t>
+        </is>
+      </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Vincient Arnold</t>
+          <t>Rafael Gonzalez</t>
         </is>
       </c>
       <c r="H121" t="inlineStr"/>
@@ -4459,17 +4572,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>At the Edge of Three Borders</t>
+          <t>Assurances Are Not Guarantees: Budapest's Lesson for Nonproliferation</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>At the Edge of Three Borders.docx</t>
+          <t>Assurances Are Not Guarantees: Budapest's Lesson for Nonproliferation.docx</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Photo Essay</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -4477,10 +4590,14 @@
           <t>geopolitics, international security</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>europe</t>
+        </is>
+      </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Emily D’Arco</t>
+          <t>Jonas Nepozitek</t>
         </is>
       </c>
       <c r="H122" t="inlineStr"/>
@@ -4491,28 +4608,33 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Assurances Are Not Guarantees: Budapest's Lesson for Nonproliferation</t>
+          <t xml:space="preserve">When Hope Invites You In For Chai
+</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Assurances Are Not Guarantees: Budapest's Lesson for Nonproliferation.docx</t>
+          <t>When hope invites you in for chai.docx</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Photo Essay</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>geopolitics, international security</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr"/>
+          <t>"human rights, humanitarian affairs, and global justice", international development, "migration, refigees, and mobility"</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>middle east</t>
+        </is>
+      </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Jonas Nepozitek</t>
+          <t>Richard Ulbricht</t>
         </is>
       </c>
       <c r="H123" t="inlineStr"/>
@@ -4523,29 +4645,33 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">When Hope Invites You In For Chai
+          <t xml:space="preserve">AI Soft Power and Korea’s Cultural Governance Model
 </t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>When hope invites you in for chai.docx</t>
+          <t>AI Soft Power and Korea’s Cultural Governance Model.docx</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Photo Essay</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>"human rights, humanitarian affairs, and global justice", international development, "migration, refigees, and mobility"</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr"/>
+          <t>"governance, democracy, and institutions", social innovation</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>east asia</t>
+        </is>
+      </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Kevin Chen</t>
+          <t>Rachel Lee</t>
         </is>
       </c>
       <c r="H124" t="inlineStr"/>
@@ -4556,13 +4682,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">AI Soft Power and Korea’s Cultural Governance Model
-</t>
+          <t>Recruiting Global Talent: Japan’s Higher Education amid a New Wave of Conservatism</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>AI Soft Power and Korea’s Cultural Governance Model.docx</t>
+          <t>Recruiting Global Talent: Japan’s Higher Education amid a New Wave of Conservatism.docx</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -4572,13 +4697,17 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>"governance, democracy, and institutions", social innovation</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr"/>
+          <t>"governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice", "migration, refigees, and mobility"</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>east asia</t>
+        </is>
+      </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Mike Henry</t>
+          <t>Kevin Chen</t>
         </is>
       </c>
       <c r="H125" t="inlineStr"/>
@@ -4589,12 +4718,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Recruiting Global Talent: Japan’s Higher Education amid a New Wave of Conservatism</t>
+          <t>Beyond SAARC’s Stalemate: Minilateralism and Regional Cooperation in Asia</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Recruiting Global Talent: Japan’s Higher Education amid a New Wave of Conservatism.docx</t>
+          <t>Beyond SAARC’s Stalemate: Minilateralism and Regional Cooperation in Asia.docx</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -4604,13 +4733,17 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>"governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice", "migration, refigees, and mobility"</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr"/>
+          <t>geopolitics</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Catherine Dai</t>
+          <t>Vincient Arnold</t>
         </is>
       </c>
       <c r="H126" t="inlineStr"/>
@@ -4621,28 +4754,33 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Beyond SAARC’s Stalemate: Minilateralism and Regional Cooperation in Asia</t>
+          <t xml:space="preserve">Beyond Survival: How Korean Concepts of Wellbeing Challenge Patient-Centered Cancer Care
+</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Beyond SAARC’s Stalemate: Minilateralism and Regional Cooperation in Asia.docx</t>
+          <t>Beyond Survival: How Korean Concepts of Wellbeing Challenge Patient-Centered Cancer Care.docx</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>geopolitics</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr"/>
+          <t>global health</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>east asia</t>
+        </is>
+      </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Michael Iwuoha</t>
+          <t>Catherine Dai</t>
         </is>
       </c>
       <c r="H127" t="inlineStr"/>
@@ -4653,29 +4791,32 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyond Survival: How Korean Concepts of Wellbeing Challenge Patient-Centered Cancer Care
-</t>
+          <t xml:space="preserve">The Limits of the Brussels Effect in a Multipolar World: Why EU Regulatory Power Meets Resistance from Emerging Economies </t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Beyond Survival: How Korean Concepts of Wellbeing Challenge Patient-Centered Cancer Care.docx</t>
+          <t>The Limits of the Brussels Effect in a Multipolar World: Why EU Regulatory Power Meets Resistance from Emerging Economies .docx</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Book Review</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>global health</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr"/>
+          <t>"global economy, finance, and trade"</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>europe</t>
+        </is>
+      </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Mike Henry</t>
+          <t>Gabriel Falk</t>
         </is>
       </c>
       <c r="H128" t="inlineStr"/>
@@ -4686,28 +4827,32 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Limits of the Brussels Effect in a Multipolar World: Why EU Regulatory Power Meets Resistance from Emerging Economies </t>
+          <t>Optimizing for Impact: A Data-Driven Roadmap to Strengthen Health Systems and Achieve UHC in LMICs</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>The Limits of the Brussels Effect in a Multipolar World: Why EU Regulatory Power Meets Resistance from Emerging Economies .docx</t>
+          <t>Optimizing for Impact: A Data-Driven Roadmap to Strengthen Health Systems and Achieve UHC in LMICs.docx</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Book Review</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>"global economy, finance, and trade"</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr"/>
+          <t>global health</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Rachel Lee</t>
+          <t>Mike Henry</t>
         </is>
       </c>
       <c r="H129" t="inlineStr"/>
@@ -4718,12 +4863,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Optimizing for Impact: A Data-Driven Roadmap to Strengthen Health Systems and Achieve UHC in LMICs</t>
+          <t>Integrating ‘Upstream and Overlooked’ Afghanistan into Central Asia's Water Future</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Optimizing for Impact: A Data-Driven Roadmap to Strengthen Health Systems and Achieve UHC in LMICs.docx</t>
+          <t>Integrating ‘Upstream and Overlooked’ Afghanistan into Central Asia's Water Future.docx</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -4733,13 +4878,18 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>global health</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr"/>
+          <t>"governance, democracy, and institutions", other</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>south asia
+central asia</t>
+        </is>
+      </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Catherine Dai</t>
+          <t>Emily D’Arco</t>
         </is>
       </c>
       <c r="H130" t="inlineStr"/>
@@ -4750,28 +4900,32 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Integrating ‘Upstream and Overlooked’ Afghanistan into Central Asia's Water Future</t>
+          <t>Does the Revolution Live in Viet Nam?: From City to Countryside, the Party Flag Flies</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Integrating ‘Upstream and Overlooked’ Afghanistan into Central Asia's Water Future.docx</t>
+          <t>Does the Revolution Live in Viet Nam?: From City to Countryside, the Party Flag Flies.docx</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Photo Essay</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>"governance, democracy, and institutions", other</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr"/>
+          <t>"global economy, finance, and trade", "governance, democracy, and institutions"</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>southeast asia</t>
+        </is>
+      </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Gabriel Falk</t>
+          <t>Sarah Cheung</t>
         </is>
       </c>
       <c r="H131" t="inlineStr"/>
@@ -4782,28 +4936,32 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Does the Revolution Live in Viet Nam?: From City to Countryside, the Party Flag Flies</t>
+          <t>Inheritance Rights for Women in Morocco: Bypassing Legal Constraints Through Social Policy</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Does the Revolution Live in Viet Nam?: From City to Countryside, the Party Flag Flies.docx</t>
+          <t>Inheritance Rights for Women in Morocco: Bypassing Legal Constraints Through Social Policy.docx</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Photo Essay</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>"global economy, finance, and trade", "governance, democracy, and institutions"</t>
-        </is>
-      </c>
-      <c r="F132" t="inlineStr"/>
+          <t>international development, social innovation</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>middle east</t>
+        </is>
+      </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Jacob Coughlin</t>
+          <t>Michael Iwuoha</t>
         </is>
       </c>
       <c r="H132" t="inlineStr"/>
@@ -4814,28 +4972,32 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Inheritance Rights for Women in Morocco: Bypassing Legal Constraints Through Social Policy</t>
+          <t>Rethinking Corruption: What Afghanistan Reveals About Cash Assistance</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Inheritance Rights for Women in Morocco: Bypassing Legal Constraints Through Social Policy.docx</t>
+          <t>Rethinking Corruption: What Afghanistan Reveals About Cash Assistance.docx</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>international development, social innovation</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr"/>
+          <t>"human rights, humanitarian affairs, and global justice", international development</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Sarah Cheung</t>
+          <t>Lisa de Rafols</t>
         </is>
       </c>
       <c r="H133" t="inlineStr"/>
@@ -4846,28 +5008,32 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Rethinking Corruption: What Afghanistan Reveals About Cash Assistance</t>
+          <t>Diego Garcia Will Be A Key Asset For Antarctic Struggle</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Rethinking Corruption: What Afghanistan Reveals About Cash Assistance.docx</t>
+          <t>Diego Garcia will be a key asset for Antarctic struggle.docx</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Op-Ed</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>"human rights, humanitarian affairs, and global justice", international development</t>
-        </is>
-      </c>
-      <c r="F134" t="inlineStr"/>
+          <t>geopolitics, "peace and conflict, peacebuilding"</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Lisa de Rafols</t>
+          <t>Rafael Gonzalez</t>
         </is>
       </c>
       <c r="H134" t="inlineStr"/>
@@ -4878,12 +5044,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Diego Garcia Will Be A Key Asset For Antarctic Struggle</t>
+          <t>To the Delight of Populist Strongmen: Judicial Anti-Institutionalism in Turkey and the United States</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Diego Garcia will be a key asset for Antarctic struggle.docx</t>
+          <t>To the Delight of Populist Strongmen: Judicial Anti-Institutionalism in Turkey and the United States.docx</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -4893,13 +5059,17 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>geopolitics, "peace and conflict, peacebuilding"</t>
-        </is>
-      </c>
-      <c r="F135" t="inlineStr"/>
+          <t>"diplomacy, leadership, and foreign policy", "governance, democracy, and institutions"</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>Richard Ulbricht</t>
+          <t>Jacob Coughlin</t>
         </is>
       </c>
       <c r="H135" t="inlineStr"/>
@@ -4910,28 +5080,32 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>To the Delight of Populist Strongmen: Judicial Anti-Institutionalism in Turkey and the United States</t>
+          <t>India–EU Free Trade Agreement: Partnership, or Regulatory Power Play?</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>To the Delight of Populist Strongmen: Judicial Anti-Institutionalism in Turkey and the United States.docx</t>
+          <t>India–EU Free Trade Agreement: Partnership, or Regulatory Power Play?.docx</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Op-Ed</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>"diplomacy, leadership, and foreign policy", "governance, democracy, and institutions"</t>
-        </is>
-      </c>
-      <c r="F136" t="inlineStr"/>
+          <t>geopolitics, "global economy, finance, and trade", international development, international law, international security</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Rafael Gonzalez</t>
+          <t>Rachel Lee</t>
         </is>
       </c>
       <c r="H136" t="inlineStr"/>
@@ -4942,12 +5116,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>How People to people Diplomacy Is About Democracy</t>
+          <t>Balancing On A Knife’s Edge: Southeast Asia’s Strategic Gamble</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>How People To People Diplomacy Is About Democracy.docx</t>
+          <t>Balancing On A Knife’s Edge: Southeast Asia’s Strategic Gamble.docx</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -4957,16 +5131,2376 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>southeast asia</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Sarah Cheung</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Parallel Media Wars - Media Ethics, Disinformation &amp; the India-Pakistan Crisis</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Parallel Media Wars - Media Ethics, Disinformation &amp; the India-Pakistan Crisis.docx</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>"peace and conflict, peacebuilding", "technology, cybersecurity, and data governance"</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Richard Ulbricht</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Of Digital Sovereignty in Civilian and Military AI - Europe’s quest towards independence in and hybridisation of civilian-military AI systems</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Of Digital Sovereignty in Civilian and Military AI - Europe’s quest towards independence in and hybridisation of civilian-military AI systems.docx</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>geopolitics, "technology, cybersecurity, and data governance"</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>europe</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Jonas Nepozitek</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>China’s Missile Force, and What To Make of Its Strides</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>China’s Missile Force, and What To Make of Its Strides.docx</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>geopolitics, international security</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>east asia</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Kevin Chen</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>The International Diplomacy over Rare Earth Elements(REEs): A confluence of the new era of Geo-Politics and International Trade</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>The International Diplomacy over Rare Earth Elements(REEs): A confluence of the new era of Geo-Politics and International Trade.docx</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>east asia</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Rachel Lee</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Oil, Gold, and the Structural Repositioning of American Supremacy</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Oil, Gold, and the Structural Repositioning of American Supremacy.docx</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics, "governance, democracy, and institutions", international security, "peace and conflict, peacebuilding"</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>north america</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Gabriel Falk</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>When Youth Outruns The State - Demography, Digital Power, and the Political Econonmy of Tolerance in India</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>When Youth Outruns The State - Demography, Digital Power, and the Political Econonmy of Tolerance in India.docx</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>"governance, democracy, and institutions"</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Richard Ulbricht</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">India’s Quiet Territorial Strategy in the Eastern Himalayas
+</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>India’s Quiet Territorial Strategy in the Eastern Himalayas.docx</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>geopolitics, international security</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Vincient Arnold</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Venezuela and the Transactional Turn in Geopolitics: Why the U.S. Intervention Signals the End of Stable Multipolar Equilibrium</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Venezuela and the Transactional Turn in Geopolitics: Why the U.S. Intervention Signals the End of Stable Multipolar Equilibrium.docx</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>geopolitics</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>latin america</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Michael Iwuoha</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>The Predictability Paradox of AI Governance: Why States Regulate Technology After Harm</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>The Predictability Paradox of AI Governance: Why States Regulate Technology After Harm.docx</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>"governance, democracy, and institutions", "technology, cybersecurity, and data governance"</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Emily D’Arco</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Who Protects the People When the State Becomes the Threat? -
+Human security vulnerabilities facing girls and women in Georgia</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Who Protects the People When the State Becomes the Threat? - Human security vulnerabilities facing girls and women in Georgia.docx</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>"human rights, humanitarian affairs, and global justice"</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>central asia/eurasia</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Catherine Dai</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How the US, Global South, and Neutral Bystanders Shape a New Geopolitical Order
+</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>How the US, Global South, and Neutral Bystanders  Shape a New Geopolitical Order.docx</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>geopolitics, "technology, cybersecurity, and data governance"</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Mike Henry</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>From Rule-Takers to Regulatory Entrepreneurs: Expanding Global Majority Agency in AI Governanc</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>From Rule-Takers to Regulatory Entrepreneurs: Expanding Global Majority Agency in AI Governanc.docx</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>"governance, democracy, and institutions", "technology, cybersecurity, and data governance"</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Lisa de Rafols</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Blacking Out Rights: Internet Shutdowns and Digital Free Expression</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Blacking Out Rights:  Internet Shutdowns and Digital Free Expression.docx</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>"human rights, humanitarian affairs, and global justice"</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Jacob Coughlin</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Climate Displacement and the Failure of International Refugee Law: A Policy Blueprint for Global Protection</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Climate Displacement and the Failure of International Refugee Law: A Policy Blueprint for Global Protection.docx</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>"climate, energy, and sustainability", "human rights, humanitarian affairs, and global justice", international law</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Emily D’Arco</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Self-Undermining Logic of Breaking International Norms: 
+An American Case Study
+</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>The Self-Undermining Logic of Breaking International Norms:  An American Case Study.docx</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>international security</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Jonas Nepozitek</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Method of Deeds: Stewardship in Regions of Unsettled Heritage
+A Model for Post-Conflict Reconciliation and Cultural Diplomacy
+</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>The Method of Deeds: Stewardship in Regions of Unsettled Heritage A Model for Post-Conflict Reconciliation and Cultural Diplomacy.docx</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy"</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>europe</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Gabriel Falk</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>China’s Anti-Communist</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>China’s Anti-Communist.docx</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>"technology, cybersecurity, and data governance", "human rights, humanitarian affairs, and global justice", social innovation</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>east asia</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Kevin Chen</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Climate Displacement as a Shared Regional Responsibility in the Bay of Bengal</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Climate Displacement as a Shared Regional Responsibility in the Bay of Bengal.docx</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>"climate, energy, and sustainability", "migration, refigees, and mobility"</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Rafael Gonzalez</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Things the Rush Conceals</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Climate Displacement as a Shared Regional Responsibility in the Bay of Bengal.docx</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Photo Essay</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>"human rights, humanitarian affairs, and global justice"</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Richard Ulbricht</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Operation Sindoor and Hindu nation: Women’s bodies in Hindu nationalist politics</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Operation Sindoor and Hindu nation: Women’s bodies in Hindu nationalist politics.docx</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>"governance, democracy, and institutions", "peace and conflict, peacebuilding"</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Vincient Arnold</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Securitization of Submarine Cables - How Southeast Asian countries navigate through the US-China undersea cable race in the region</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Securitization of Submarine Cables - How Southeast Asian countries navigate through the US-China undersea cable race in the region.docx</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>geopolitics</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>southeast asia</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Sarah Cheung</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Between Us and Them: The Role of Italian Media Narratives as a Bordering Agent</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Between Us and Them:  The Role of Italian Media Narratives as a Bordering Agent.docx</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>"governance, democracy, and institutions", "migration, refigees, and mobility"</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>europe</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Jonas Nepozitek</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Growth Without Guarantees: How Global Cities Normalize Economic Insecurity</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Growth Without Guarantees: How Global Cities Normalize Economic Insecurity.docx</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Photo Essay</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>"global economy, finance, and trade", international development, international security</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Mike Henry</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Book Review "Bikolpo Arthanity"</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Book Review "Bikolpo Arthanity".docx</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Book Review</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>"peace and conflict, peacebuilding", "human rights, humanitarian affairs, and global justice", "governance, democracy, and institutions", "climate, energy, and sustainability"</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Lisa de Rafols</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Has India’s Maoist Insurgency Entered Its Terminal Phase?</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Has India’s Maoist Insurgency Entered Its Terminal Phase?.docx</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>"governance, democracy, and institutions", geopolitics, "peace and conflict, peacebuilding"</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Jacob Coughlin</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Comity for the Empty Shell: Structural Subordination, Sovereign Ring-Fencing, and the Limits of the Model Law in China's Evergrande Crisis.</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Comity for the Empty Shell: Structural Subordination, Sovereign Ring-Fencing, and the Limits of the Model Law in China's Evergrande Crisis..docx</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>"global economy, finance, and trade", international law</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Rachel Lee</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>The Invisible Frontline: Undersea Internet Cables and the Future of Geopolitical Conflict</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>The Invisible Frontline: Undersea Internet Cables and the Future of Geopolitical Conflict.docx</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy"</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Emily D’Arco</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>The High Seas Treaty: A Historic Breakthrough or Hollow Promise?</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>The High Seas Treaty: A Historic Breakthrough or Hollow Promise?.docx</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>"climate, energy, and sustainability"</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Michael Iwuoha</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Fragmented Order: How Minilateral Coalitions Are Rewiring—Not Replacing—Multilateralism</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Fragmented Order: How Minilateral Coalitions Are Rewiring—Not Replacing—Multilateralism .docx</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>united nations and multilateral institutions</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Mike Henry</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Masterstroke Mirage: India’s Diplomatic Triumphs, Rhetoric, and Regional Reality</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Masterstroke Mirage: India’s Diplomatic Triumphs, Rhetoric, and Regional Reality.docx</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics, "global economy, finance, and trade"</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Rafael Gonzalez</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">“Utility Over Universality: The Quiet Erosion of Liberal Internationalism”
+</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>“Utility Over Universality: The Quiet Erosion of Liberal Internationalism”.docx</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
           <t>"diplomacy, leadership, and foreign policy", "governance, democracy, and institutions"</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr"/>
-      <c r="G137" t="inlineStr">
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>north america</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Kevin Chen</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>How can President Trump bring Lasting Peace to the Korean Peninsula</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>How can President Trump bring Lasting Peace to the Korean Peninsula?.docx</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy", "governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice", international security</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>north america
+east asia</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
         <is>
           <t>Vincient Arnold</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
+      <c r="H169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>The IMF’s Repeat-Customer Problem</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>The IMF’s Repeat-Customer Problem.docx</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>"global economy, finance, and trade", "governance, democracy, and institutions", international development</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Sarah Cheung</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Counter-Terrorism Policy in the European Union:
+Successes, Failures, and Room for Improvement
+</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Counter-Terrorism Policy in the European Union: Successes, Failures, and Room for Improvement.docx</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>international law, international security</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>north america</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Hekmat Aboukhater</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Weaponized Interdependence in Rare Earth Diplomacy: The U.S.–China Competition and Central Asia</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Weaponized Interdependence in Rare Earth Diplomacy: The U.S.–China Competition and Central Asia.docx</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>geopolitics, "global economy, finance, and trade", international development</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Lisa de Rafols</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>When Survival Becomes Conditional - The Falepili Union and the Future of Climate Displacement</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>When Survival Becomes Conditional - The Falepili Union and the Future of Climate Displacement.docx</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>"climate, energy, and sustainability", "migration, refigees, and mobility"</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>oceania and the pacific</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Richard Ulbricht</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>The Political Economy of AI Adoption in Security Governance</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>The Political Economy of AI Adoption in Security Governance.docx</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>"governance, democracy, and institutions", "technology, cybersecurity, and data governance"</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>north america</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Catherine Dai</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Cross-arctic Biodiversity Research Networks are Becoming History: We Have to Record Them While We Still Can</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Cross-arctic Biodiversity Research Networks are Becoming History: We Have to Record Them While We Still Can.docx</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>"climate, energy, and sustainability", "diplomacy, leadership, and foreign policy", geopolitics</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>central asia/eurasia</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Gabriel Falk</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Abandoning Neutrality: Why Sweden Joined NATO in 2024</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Abandoning Neutrality: Why Sweden Joined NATO in 2024.docx</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy", international security</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>europe</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Jonas Nepozitek</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Has South Asia Escaped India’s Imagination?</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Has South Asia Escaped India’s Imagination?.docx</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Jacob Coughlin</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>South Asia in Crisis, or No South Asia?</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>South Asia in Crisis, or No South Asia?.docx</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>geopolitics</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Rachel Lee</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transnational Crime: A Shaper of International Relations
+</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Transnational Crime: A Shaper of International Relations.docx</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>international security, "peace and conflict, peacebuilding"</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Emily D’Arco</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Party-In-The-Loop: Acceptable Autonomy in the PLA</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Party-In-The-Loop: Acceptable Autonomy in the PLA.docx</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>geopolitics, international security</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>east asia</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Kevin Chen</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Judicial Independence and the Future of Climate Justice</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Judicial Independence and the Future of Climate Justice.docx</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>"climate, energy, and sustainability", "governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice"</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>latin america</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Michael Iwuoha</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>At Least US Protectionism Is Honest</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>At Least US Protectionism Is Honest.docx</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>"climate, energy, and sustainability", "diplomacy, leadership, and foreign policy", "global economy, finance, and trade"</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Mike Henry</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Contemporary Economic Statecraft: The Efficacy of Sanctions</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Contemporary Economic Statecraft: The Efficacy of Sanctions.docx</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics, "global economy, finance, and trade"</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Sarah Cheung</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Life Inside Venezuela, an Unfinished Petrostate</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Life Inside Venezuela, an Unfinished Petrostate.docx</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Photo Essay</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>"global economy, finance, and trade", "governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice"</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>latin america</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Alexandra Helfgott</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>A Year of Rare Earth Elements</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>A Year of Rare Earth Elements.docx</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>"climate, energy, and sustainability", "diplomacy, leadership, and foreign policy", geopolitics, international law, international security, "technology, cybersecurity, and data governance"</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Lisa de Rafols</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Sharpening the Spears of Long-Term Sustainability as a Legal Principle in the New Space Age</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Sharpening the Spears of Long-Term Sustainability as a Legal Principle in the New Space Age.docx</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>international law</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Michael Iwuoha</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Fault lines in Bangladesh’s political journey toward democracy</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Fault lines in Bangladesh’s political journey toward democracy.docx</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>"governance, democracy, and institutions"</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Rafael Gonzalez</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Price of Market Access: Carbon, Competitiveness, and EU-India Trade
+</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>The Price of Market Access: Carbon, Competitiveness, and EU-India Trade.docx</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>"climate, energy, and sustainability", "global economy, finance, and trade"</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Gabriel Falk</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Slowing the Pentagon’s Revolving Door - Why Special Interests Quietly Override National Security Interests</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Slowing the Pentagon’s Revolving Door - Why Special Interests Quietly Override National Security Interests.docx</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>"governance, democracy, and institutions"</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>north america</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Hekmat Aboukhater</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Huntington, Historical Ethos of a Superpower and the Way Out</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Huntington, Historical Ethos of a Superpower and the Way Out.docx</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Jacob Coughlin</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marines and Submarines: A Recipe for Sea Denial in the First Island Chain
+</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Marines and Submarines: A Recipe for Sea Denial in the First Island Chain.docx</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>geopolitics, international security</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>north america</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Catherine Dai</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Democracy's Gatekeeper: Why Failure of Legal Constraints is Necessary for Democratic Backsliding </t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Op-Ed - Democracy.docx</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>"governance, democracy, and institutions"</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Rachel Lee</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>When Trade Stops Tying Hands: The Fragmentation of Economic Peace</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>When Trade Stops Tying Hands: The Fragmentation of Economic Peace.docx</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>geopolitics, "global economy, finance, and trade", international development</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Emily D’Arco</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Digital Payment System is the Missing Key to Gaza’s Reconstruction</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Digital Payment System is the Missing Key to Gaza’s Reconstruction.docx</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>"global economy, finance, and trade", "peace and conflict, peacebuilding"</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>middle east</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Hekmat Aboukhater</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>The Right to Strike in China, Legal Absence and Practical Persistence</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>The Right to Strike in China, Legal Absence and Practical Persistence.docx</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>"governance, democracy, and institutions", "human rights, humanitarian affairs, and global justice"</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>east asia</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Kevin Chen</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Erosion of Mutual Vulnerability:
+Conventional counterforce and the transformation of deterrence 
+</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>The Erosion of Mutual Vulnerability: Conventional counterforce and the transformation of deterrence .docx</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>geopolitics, international security</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Jonas Nepozitek</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Energy transition: where are the women?</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Energy transition: where are the women?.docx</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>"climate, energy, and sustainability"</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Mike Henry</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Digital Public Infrastructure as Structural Soft Power</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Digital Public Infrastructure as Structural Soft Power.docx</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>"global economy, finance, and trade", "governance, democracy, and institutions", international development</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>south asia</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Richard Ulbricht</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Summit Fatigue and the Limits of Consensus</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Summit Fatigue and the Limits of Consensus.docx</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy", united nations and multilateral institutions</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Sarah Cheung</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Middle Powers on the Rise</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Middle Powers on the Rise.docx</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>geopolitics</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Jacob Coughlin</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>America Can't Stop North Korea's Nukes Without China</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>America Can't Stop North Korea's Nukes Without China.docx</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>"diplomacy, leadership, and foreign policy", geopolitics</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Gabriel Falk</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Critical Mineral, Gendered Cost</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Critical Mineral, Gendered Cost.docx</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Op-Ed</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>"climate, energy, and sustainability", geopolitics</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>cross-regional/global</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Lisa de Rafols</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>